<commit_message>
adding changes to input mult
</commit_message>
<xml_diff>
--- a/public/template_input_multiple.xlsx
+++ b/public/template_input_multiple.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Computer_Science\A_PENELITIAN\deploy trial\fe_siperad_1_trial\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2980843A-76C4-45E9-A5D1-4F9F71BA6508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C405CDA-4DC7-4EC0-85CF-9A217CBC58B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Angkatan" sheetId="1" r:id="rId1"/>
@@ -27,10 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
-  <si>
-    <t>nama_alat</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>stok</t>
   </si>
@@ -59,12 +56,6 @@
     <t>jam</t>
   </si>
   <si>
-    <t>status_alat</t>
-  </si>
-  <si>
-    <t>0 = tidak tersedia</t>
-  </si>
-  <si>
     <t>1 = tersedia</t>
   </si>
   <si>
@@ -99,6 +90,12 @@
   </si>
   <si>
     <t>kelas</t>
+  </si>
+  <si>
+    <t>deskripsi_barang</t>
+  </si>
+  <si>
+    <t>nama_barang</t>
   </si>
 </sst>
 </file>
@@ -484,7 +481,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -502,31 +499,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>20</v>
-      </c>
-      <c r="H1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -536,36 +533,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -583,28 +565,28 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -622,7 +604,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -640,7 +622,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -658,7 +640,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -676,13 +658,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" t="s">
-        <v>7</v>
-      </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>